<commit_message>
Evento #1 registrado en reporte_2026-05-29.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-05-29.xlsx
+++ b/datos/excel/reporte_2026-05-29.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,51 @@
         <v>69</v>
       </c>
       <c r="K2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00:01:39</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>320.31</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-20.28</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>609.4 Hz | 914.1 Hz | 1257.8 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2502</v>
+      </c>
+      <c r="J3" t="n">
+        <v>11839</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Evento #2 registrado en reporte_2026-05-29.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-05-29.xlsx
+++ b/datos/excel/reporte_2026-05-29.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +605,51 @@
       <c r="K4" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>00:03:34</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>468.75</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-22.39</v>
+      </c>
+      <c r="G5" t="n">
+        <v>99.98</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>937.5 Hz | 1421.9 Hz | 1851.6 Hz</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>2514</v>
+      </c>
+      <c r="J5" t="n">
+        <v>73</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>🚨 SÍ</t>
         </is>
       </c>
     </row>

</xml_diff>